<commit_message>
Refactor proposal-tldr and research documentation; update realization events in technical spec
- Updated charitable transfer treatment in proposal-tldr to reflect realization events as of Aug 2026.
- Added weekly briefing updates in research.md regarding Prop 40 status and STEP Act legislation.
- Revised realization events in technical_spec.md to include leveraging appreciated assets and removed charitable exception.
- Clarified charitable donation treatment to align with new realization rules, detailing tax implications and subsidy calculations.
</commit_message>
<xml_diff>
--- a/internal/analysis/calibration_comparison.xlsx
+++ b/internal/analysis/calibration_comparison.xlsx
@@ -642,6 +642,7 @@
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -682,6 +683,12 @@
 $1.25M–$4M</t>
         </is>
       </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>New Lower
+$1M–$3M</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -704,6 +711,11 @@
           <t>$1.25M</t>
         </is>
       </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>$1M</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -726,6 +738,11 @@
           <t>$2.5M</t>
         </is>
       </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>$2M</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -748,6 +765,11 @@
           <t>$4M</t>
         </is>
       </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>$3M</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -770,6 +792,11 @@
           <t>$2.75M</t>
         </is>
       </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>$2M</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -792,6 +819,11 @@
           <t>~$7.4M</t>
         </is>
       </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>~$5.6M</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -814,6 +846,11 @@
           <t>+$70-200B</t>
         </is>
       </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>+$75-210B (est.)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -836,6 +873,11 @@
           <t>~3-5%</t>
         </is>
       </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>~6-10% (est.)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -858,6 +900,11 @@
           <t>$6.06M (pays $1.54M more)</t>
         </is>
       </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>$6.29M (pays $1.77M more)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -880,6 +927,11 @@
           <t>$34.2M (+$11.6M)</t>
         </is>
       </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>$34.41M (+$11.8M)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -902,6 +954,11 @@
           <t>Lowest</t>
         </is>
       </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -924,6 +981,11 @@
           <t>Strongest</t>
         </is>
       </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Strongest</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -944,6 +1006,11 @@
       <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Most affected filers</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Most affected (below Aggressive)</t>
         </is>
       </c>
     </row>
@@ -973,6 +1040,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1020,6 +1088,11 @@
         </is>
       </c>
       <c r="G5" s="41" t="n"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>New Lower</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -1039,6 +1112,9 @@
         <v>1250000</v>
       </c>
       <c r="G6" s="41" t="n"/>
+      <c r="H6" s="13" t="n">
+        <v>1000000</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -1058,6 +1134,9 @@
         <v>4000000</v>
       </c>
       <c r="G7" s="41" t="n"/>
+      <c r="H7" s="13" t="n">
+        <v>3000000</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -1077,6 +1156,9 @@
         <v>2500000</v>
       </c>
       <c r="G8" s="41" t="n"/>
+      <c r="H8" s="13" t="n">
+        <v>2000000</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -1096,6 +1178,9 @@
         <v>8000000</v>
       </c>
       <c r="G9" s="41" t="n"/>
+      <c r="H9" s="13" t="n">
+        <v>6000000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -1115,6 +1200,9 @@
         <v>2750000</v>
       </c>
       <c r="G10" s="41" t="n"/>
+      <c r="H10" s="13" t="n">
+        <v>2000000</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -1134,6 +1222,9 @@
         <v>7357955</v>
       </c>
       <c r="G11" s="41" t="n"/>
+      <c r="H11" s="13" t="n">
+        <v>5606061</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
@@ -1154,6 +1245,11 @@
       <c r="F13" s="16" t="inlineStr">
         <is>
           <t>~3-5%</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>~6-10% (est.)</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1211,6 +1307,8 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1271,6 +1369,16 @@
           <t>Aggressive Eff. Rate</t>
         </is>
       </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Lower Tax</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Lower Eff. Rate</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1305,6 +1413,12 @@
       <c r="J4" s="18" t="n">
         <v>0</v>
       </c>
+      <c r="K4" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1339,6 +1453,12 @@
       <c r="J5" s="18" t="n">
         <v>0.0577</v>
       </c>
+      <c r="K5" s="19" t="n">
+        <v>299700</v>
+      </c>
+      <c r="L5" s="18" t="n">
+        <v>0.107</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1373,6 +1493,12 @@
       <c r="J6" s="18" t="n">
         <v>0.3189</v>
       </c>
+      <c r="K6" s="20" t="n">
+        <v>6290000</v>
+      </c>
+      <c r="L6" s="18" t="n">
+        <v>0.3311</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1407,6 +1533,12 @@
       <c r="J7" s="18" t="n">
         <v>0.3598</v>
       </c>
+      <c r="K7" s="20" t="n">
+        <v>34410000</v>
+      </c>
+      <c r="L7" s="18" t="n">
+        <v>0.3622</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1441,6 +1573,12 @@
       <c r="J8" s="18" t="n">
         <v>0.3053</v>
       </c>
+      <c r="K8" s="20" t="n">
+        <v>4810000</v>
+      </c>
+      <c r="L8" s="18" t="n">
+        <v>0.3207</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1475,6 +1613,12 @@
       <c r="J9" s="18" t="n">
         <v>0.37</v>
       </c>
+      <c r="K9" s="20" t="n">
+        <v>1850000</v>
+      </c>
+      <c r="L9" s="18" t="n">
+        <v>0.37</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1507,6 +1651,12 @@
         <v>148000000</v>
       </c>
       <c r="J10" s="18" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="K10" s="20" t="n">
+        <v>148000000</v>
+      </c>
+      <c r="L10" s="18" t="n">
         <v>0.37</v>
       </c>
     </row>
@@ -1549,6 +1699,9 @@
         <v>0</v>
       </c>
       <c r="J13" s="14" t="n"/>
+      <c r="K13" s="22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -1573,6 +1726,9 @@
         <v>-393377</v>
       </c>
       <c r="J14" s="14" t="n"/>
+      <c r="K14" s="23" t="n">
+        <v>-255300</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -1597,6 +1753,9 @@
         <v>1538750</v>
       </c>
       <c r="J15" s="14" t="n"/>
+      <c r="K15" s="24" t="n">
+        <v>1770000</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -1621,6 +1780,9 @@
         <v>11568750</v>
       </c>
       <c r="J16" s="14" t="n"/>
+      <c r="K16" s="24" t="n">
+        <v>11800000</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -1645,6 +1807,9 @@
         <v>4578750</v>
       </c>
       <c r="J17" s="14" t="n"/>
+      <c r="K17" s="24" t="n">
+        <v>4810000</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -1669,6 +1834,9 @@
         <v>1850000</v>
       </c>
       <c r="J18" s="14" t="n"/>
+      <c r="K18" s="24" t="n">
+        <v>1850000</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -1693,6 +1861,9 @@
         <v>108000000</v>
       </c>
       <c r="J19" s="14" t="n"/>
+      <c r="K19" s="24" t="n">
+        <v>108000000</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1709,7 +1880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1722,6 +1893,9 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1782,6 +1956,21 @@
           <t>Aggressive Eff. Rate</t>
         </is>
       </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Lower Rate</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Lower Tax</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Lower Eff. Rate</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="25" t="n">
@@ -1814,6 +2003,15 @@
       <c r="J4" s="18" t="n">
         <v>0</v>
       </c>
+      <c r="K4" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="25" t="n">
@@ -1846,6 +2044,15 @@
       <c r="J5" s="18" t="n">
         <v>0</v>
       </c>
+      <c r="K5" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="n">
@@ -1878,6 +2085,15 @@
       <c r="J6" s="27" t="n">
         <v>0</v>
       </c>
+      <c r="K6" s="27" t="n">
+        <v>0.0462</v>
+      </c>
+      <c r="L6" s="28" t="n">
+        <v>5781</v>
+      </c>
+      <c r="M6" s="27" t="n">
+        <v>0.0046</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="25" t="n">
@@ -1910,6 +2126,15 @@
       <c r="J7" s="18" t="n">
         <v>0.0189</v>
       </c>
+      <c r="K7" s="18" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="L7" s="17" t="n">
+        <v>92500</v>
+      </c>
+      <c r="M7" s="18" t="n">
+        <v>0.0462</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="26" t="n">
@@ -1942,6 +2167,15 @@
       <c r="J8" s="27" t="n">
         <v>0.042</v>
       </c>
+      <c r="K8" s="27" t="n">
+        <v>0.2775</v>
+      </c>
+      <c r="L8" s="28" t="n">
+        <v>208125</v>
+      </c>
+      <c r="M8" s="27" t="n">
+        <v>0.0833</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="26" t="n">
@@ -1974,6 +2208,15 @@
       <c r="J9" s="27" t="n">
         <v>0.0687</v>
       </c>
+      <c r="K9" s="27" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="L9" s="28" t="n">
+        <v>370000</v>
+      </c>
+      <c r="M9" s="27" t="n">
+        <v>0.1233</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="25" t="n">
@@ -2006,6 +2249,15 @@
       <c r="J10" s="18" t="n">
         <v>0.1757</v>
       </c>
+      <c r="K10" s="18" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="L10" s="17" t="n">
+        <v>1110000</v>
+      </c>
+      <c r="M10" s="18" t="n">
+        <v>0.222</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="25" t="n">
@@ -2038,6 +2290,15 @@
       <c r="J11" s="18" t="n">
         <v>0.2486</v>
       </c>
+      <c r="K11" s="18" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="L11" s="17" t="n">
+        <v>2220000</v>
+      </c>
+      <c r="M11" s="18" t="n">
+        <v>0.2775</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="25" t="n">
@@ -2070,6 +2331,15 @@
       <c r="J12" s="18" t="n">
         <v>0.2729</v>
       </c>
+      <c r="K12" s="18" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="L12" s="17" t="n">
+        <v>2960000</v>
+      </c>
+      <c r="M12" s="18" t="n">
+        <v>0.296</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="25" t="n">
@@ -2102,6 +2372,15 @@
       <c r="J13" s="18" t="n">
         <v>0.3053</v>
       </c>
+      <c r="K13" s="18" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="L13" s="17" t="n">
+        <v>4810000</v>
+      </c>
+      <c r="M13" s="18" t="n">
+        <v>0.3207</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="25" t="n">
@@ -2134,6 +2413,15 @@
       <c r="J14" s="18" t="n">
         <v>0.3214</v>
       </c>
+      <c r="K14" s="18" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="L14" s="17" t="n">
+        <v>6660000</v>
+      </c>
+      <c r="M14" s="18" t="n">
+        <v>0.333</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="25" t="n">
@@ -2166,6 +2454,15 @@
       <c r="J15" s="18" t="n">
         <v>0.3311</v>
       </c>
+      <c r="K15" s="18" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="L15" s="17" t="n">
+        <v>8510000</v>
+      </c>
+      <c r="M15" s="18" t="n">
+        <v>0.3404</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="25" t="n">
@@ -2198,6 +2495,15 @@
       <c r="J16" s="18" t="n">
         <v>0.3376</v>
       </c>
+      <c r="K16" s="18" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="L16" s="17" t="n">
+        <v>10360000</v>
+      </c>
+      <c r="M16" s="18" t="n">
+        <v>0.3453</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="25" t="n">
@@ -2230,6 +2536,15 @@
       <c r="J17" s="18" t="n">
         <v>0.3506</v>
       </c>
+      <c r="K17" s="18" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="L17" s="17" t="n">
+        <v>17760000</v>
+      </c>
+      <c r="M17" s="18" t="n">
+        <v>0.3552</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="25" t="n">
@@ -2261,6 +2576,15 @@
       </c>
       <c r="J18" s="18" t="n">
         <v>0.3603</v>
+      </c>
+      <c r="K18" s="18" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="L18" s="17" t="n">
+        <v>36260000</v>
+      </c>
+      <c r="M18" s="18" t="n">
+        <v>0.3626</v>
       </c>
     </row>
   </sheetData>
@@ -2278,7 +2602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2293,6 +2617,10 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2422,6 +2750,11 @@
           <t>REVENUE GAINS — AGGRESSIVE</t>
         </is>
       </c>
+      <c r="M12" s="30" t="inlineStr">
+        <is>
+          <t>REVENUE GAINS — NEW LOWER ($1M/$3M)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2484,6 +2817,26 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>Low ($B)</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>High ($B)</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -2534,6 +2887,22 @@
           <t>Same: exemption protects ordinary families either way</t>
         </is>
       </c>
+      <c r="M14" s="12" t="inlineStr">
+        <is>
+          <t>Deemed realization at death</t>
+        </is>
+      </c>
+      <c r="N14" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="O14" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="P14" s="34" t="inlineStr">
+        <is>
+          <t>Same: exemption protects ordinary families either way</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -2584,6 +2953,22 @@
           <t>Same: borrower's exemption typically exhausted</t>
         </is>
       </c>
+      <c r="M15" s="12" t="inlineStr">
+        <is>
+          <t>Buy-borrow-die closure</t>
+        </is>
+      </c>
+      <c r="N15" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="O15" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="P15" s="34" t="inlineStr">
+        <is>
+          <t>Same: borrower's exemption typically exhausted</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -2634,6 +3019,22 @@
           <t>Same: universal exemption replaces</t>
         </is>
       </c>
+      <c r="M16" s="12" t="inlineStr">
+        <is>
+          <t>QSBS elimination</t>
+        </is>
+      </c>
+      <c r="N16" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="O16" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="P16" s="34" t="inlineStr">
+        <is>
+          <t>Same: universal exemption replaces</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -2684,6 +3085,22 @@
           <t>Same: real estate flows through system</t>
         </is>
       </c>
+      <c r="M17" s="12" t="inlineStr">
+        <is>
+          <t>1031 exchange elimination</t>
+        </is>
+      </c>
+      <c r="N17" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="O17" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="P17" s="34" t="inlineStr">
+        <is>
+          <t>Same: real estate flows through system</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -2734,6 +3151,22 @@
           <t>Same: small items</t>
         </is>
       </c>
+      <c r="M18" s="12" t="inlineStr">
+        <is>
+          <t>Other preferences (OZ, 1256, etc.)</t>
+        </is>
+      </c>
+      <c r="N18" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="O18" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="P18" s="34" t="inlineStr">
+        <is>
+          <t>Same: small items</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -2784,6 +3217,22 @@
           <t>Same: contribution freeze</t>
         </is>
       </c>
+      <c r="M19" s="12" t="inlineStr">
+        <is>
+          <t>Roth reform ($5M cap)</t>
+        </is>
+      </c>
+      <c r="N19" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="O19" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="P19" s="34" t="inlineStr">
+        <is>
+          <t>Same: contribution freeze</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -2834,6 +3283,22 @@
           <t>Same: near-term shift to Roth</t>
         </is>
       </c>
+      <c r="M20" s="12" t="inlineStr">
+        <is>
+          <t>Roth acceleration (income limit removal)</t>
+        </is>
+      </c>
+      <c r="N20" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="O20" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="P20" s="34" t="inlineStr">
+        <is>
+          <t>Same: near-term shift to Roth</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="35" t="inlineStr">
@@ -2884,6 +3349,22 @@
           <t>Breakeven ~$7.4M; most gains taxed above current rates</t>
         </is>
       </c>
+      <c r="M21" s="35" t="inlineStr">
+        <is>
+          <t>Sliding scale on gains above exemption</t>
+        </is>
+      </c>
+      <c r="N21" s="35" t="n">
+        <v>37</v>
+      </c>
+      <c r="O21" s="35" t="n">
+        <v>73</v>
+      </c>
+      <c r="P21" s="36" t="inlineStr">
+        <is>
+          <t>EXTRAPOLATED from Generous/Moderate/Aggressive trend — not run through full model</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -2922,6 +3403,18 @@
         <v>293</v>
       </c>
       <c r="L22" s="37" t="n"/>
+      <c r="M22" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL GAINS</t>
+        </is>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>177</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>301</v>
+      </c>
+      <c r="P22" s="37" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
@@ -2984,14 +3477,35 @@
           <t>Directional. Range +$70B to +$200B/yr</t>
         </is>
       </c>
+      <c r="M24" s="38" t="inlineStr">
+        <is>
+          <t>NET REVENUE</t>
+        </is>
+      </c>
+      <c r="N24" s="39" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="O24" s="39" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="P24" s="40" t="inlineStr">
+        <is>
+          <t>Component math for this sheet is stale (see A2 note) — do not subtract N22-O22 minus losses. Use Summary tab: +$75-210B (est., extrapolated from the 3-point Generous/Moderate/Aggressive trend, NOT independently modeled). Recommend rebuilding full model before publishing this number.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="E12:H12"/>
     <mergeCell ref="I12:L12"/>
+    <mergeCell ref="M12:P12"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3004,8 +3518,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3042,6 +3559,11 @@
           <t>Higher 3/8</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>New Lower ($1M/$3M) — DRAFT Aug 2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3058,6 +3580,9 @@
       <c r="D5" t="n">
         <v>3000000</v>
       </c>
+      <c r="E5" t="n">
+        <v>1000000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3074,6 +3599,9 @@
       <c r="D6" t="n">
         <v>8000000</v>
       </c>
+      <c r="E6" t="n">
+        <v>3000000</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3096,6 +3624,11 @@
           <t>~$15.4M</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>~$5.6M</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3118,6 +3651,11 @@
           <t>&lt;1%</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>~6-10% (est.)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3134,6 +3672,9 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
+      <c r="E9" t="n">
+        <v>299700</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3150,6 +3691,9 @@
       <c r="D10" t="n">
         <v>5000000</v>
       </c>
+      <c r="E10" t="n">
+        <v>6290000</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3166,6 +3710,9 @@
       <c r="D11" t="n">
         <v>33120000</v>
       </c>
+      <c r="E11" t="n">
+        <v>34410000</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3188,6 +3735,11 @@
           <t>$35-160B</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>$75-210B (est.)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3210,6 +3762,11 @@
           <t>~$98B</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>~$140B (est.)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3230,6 +3787,11 @@
       <c r="D14" t="inlineStr">
         <is>
           <t>~$3-25B</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>~$37-73B (est.)</t>
         </is>
       </c>
     </row>

</xml_diff>